<commit_message>
Precios del globo Sempertex: 5" $55, 12" $127, 18" $235; mayoreo desde 12
Mayoreo: 5" $44, 12" $112 y 18" $188 a partir de 12 unidades por tamaño.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GPuHuyNqpYqoozZfmLEUUZ
</commit_message>
<xml_diff>
--- a/plantilla-productos.xlsx
+++ b/plantilla-productos.xlsx
@@ -2902,13 +2902,13 @@
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>120</v>
+        <v>44</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
@@ -2982,13 +2982,13 @@
         </is>
       </c>
       <c r="E20" s="4" t="n">
-        <v>175</v>
+        <v>127</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>155</v>
+        <v>112</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
@@ -3062,13 +3062,13 @@
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>265</v>
+        <v>235</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>240</v>
+        <v>188</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Productos con tamaños: el código de sus filas fija el enlace
Las filas de un producto con varios tamaños llevan el mismo código, que
se usa como enlace del producto (si se renombra, el enlace y los carritos
no cambian). Si las filas traen códigos distintos se usa el primero y se
avisa en la página de revisión.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GPuHuyNqpYqoozZfmLEUUZ
</commit_message>
<xml_diff>
--- a/plantilla-productos.xlsx
+++ b/plantilla-productos.xlsx
@@ -946,7 +946,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Identificador para el enlace del producto. Opcional: si lo dejas vacío se crea con el nombre. No lo cambies una vez publicado, porque lo usan los carritos y los enlaces compartidos.
+        <t>Identificador para el enlace del producto. Opcional: si lo dejas vacío se crea con el nombre. No lo cambies una vez publicado, porque lo usan los carritos y los enlaces compartidos. En un producto con varios tamaños, pon el mismo código en todas sus filas.
 Ejemplo: globo-foil-estrella-18</t>
       </text>
     </comment>
@@ -2885,7 +2885,11 @@
       <c r="V18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n"/>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>globo-sempertex-redondo</t>
+        </is>
+      </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Globo Sempertex redondo</t>
@@ -2965,7 +2969,11 @@
       <c r="V19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n"/>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>globo-sempertex-redondo</t>
+        </is>
+      </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Globo Sempertex redondo</t>
@@ -3045,7 +3053,11 @@
       <c r="V20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>globo-sempertex-redondo</t>
+        </is>
+      </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Globo Sempertex redondo</t>
@@ -6456,7 +6468,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="45" customHeight="1">
+    <row r="37" ht="60" customHeight="1">
       <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Código</t>
@@ -6464,7 +6476,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Identificador para el enlace del producto. Opcional: si lo dejas vacío se crea con el nombre. No lo cambies una vez publicado, porque lo usan los carritos y los enlaces compartidos.</t>
+          <t>Identificador para el enlace del producto. Opcional: si lo dejas vacío se crea con el nombre. No lo cambies una vez publicado, porque lo usan los carritos y los enlaces compartidos. En un producto con varios tamaños, pon el mismo código en todas sus filas.</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Sempertex: logo de la marca, sección Globos Sempertex y Reflex con sus presentaciones
- Logo de Sempertex en el menú, la portada, las tarjetas, la página del
  producto y su ficha, y nueva sección #/marca/sempertex.
- Globo Sempertex Reflex como producto aparte: 5" y 12" (50 pz) y 18" en
  bolsas de 15 y 25 pz, con mayoreo desde 12 bolsas.
- La bolsa de 5" del Sempertex redondo ahora es de 50 piezas.
- Plantilla y README actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GPuHuyNqpYqoozZfmLEUUZ
</commit_message>
<xml_diff>
--- a/plantilla-productos.xlsx
+++ b/plantilla-productos.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carta Sempertex" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Productos'!$A$1:$V$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Productos'!$A$1:$V$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1369,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V59"/>
+  <dimension ref="A1:V63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2916,25 +2916,25 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>bolsa con 100 piezas</t>
+          <t>bolsa con 50 piezas</t>
         </is>
       </c>
       <c r="I19" s="3" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Globo redondo de látex Sempertex con colores firmes y acabado parejo. Elige el tono en la carta de colores y el tamaño: 5" para arcos orgánicos y rellenos, 12" para decoración en general y 18" para dar volumen.</t>
+          <t>Globo redondo de látex Sempertex con colores firmes y acabado parejo. Elige el tono en la carta de colores y el tamaño: 5" para arcos orgánicos y rellenos, 12" para decoración en general y 18" para dar volumen. El acabado espejo está en el Globo Sempertex Reflex.</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>Marca: Sempertex; Forma: Redondo; Material: Látex natural; Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 85, en 8 familias: Fashion, Pastel Mate, Neón, Pastel Dusk, Satín, Silk, Metálico y Reflex</t>
+          <t>Marca: Sempertex; Forma: Redondo; Material: Látex natural; Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 74, en 7 familias: Fashion, Pastel Mate, Neón, Pastel Dusk, Satín, Silk y Metálico</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>Carta Sempertex</t>
+          <t>Sempertex Fashion, Sempertex Pastel Mate, Sempertex Neón, Sempertex Pastel Dusk, Sempertex Satín, Sempertex Silk, Sempertex Metálico</t>
         </is>
       </c>
       <c r="M19" s="3" t="n"/>
@@ -3008,17 +3008,17 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Globo redondo de látex Sempertex con colores firmes y acabado parejo. Elige el tono en la carta de colores y el tamaño: 5" para arcos orgánicos y rellenos, 12" para decoración en general y 18" para dar volumen.</t>
+          <t>Globo redondo de látex Sempertex con colores firmes y acabado parejo. Elige el tono en la carta de colores y el tamaño: 5" para arcos orgánicos y rellenos, 12" para decoración en general y 18" para dar volumen. El acabado espejo está en el Globo Sempertex Reflex.</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Marca: Sempertex; Forma: Redondo; Material: Látex natural; Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 85, en 8 familias: Fashion, Pastel Mate, Neón, Pastel Dusk, Satín, Silk, Metálico y Reflex</t>
+          <t>Marca: Sempertex; Forma: Redondo; Material: Látex natural; Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 74, en 7 familias: Fashion, Pastel Mate, Neón, Pastel Dusk, Satín, Silk y Metálico</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>Carta Sempertex</t>
+          <t>Sempertex Fashion, Sempertex Pastel Mate, Sempertex Neón, Sempertex Pastel Dusk, Sempertex Satín, Sempertex Silk, Sempertex Metálico</t>
         </is>
       </c>
       <c r="M20" s="3" t="n"/>
@@ -3092,17 +3092,17 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Globo redondo de látex Sempertex con colores firmes y acabado parejo. Elige el tono en la carta de colores y el tamaño: 5" para arcos orgánicos y rellenos, 12" para decoración en general y 18" para dar volumen.</t>
+          <t>Globo redondo de látex Sempertex con colores firmes y acabado parejo. Elige el tono en la carta de colores y el tamaño: 5" para arcos orgánicos y rellenos, 12" para decoración en general y 18" para dar volumen. El acabado espejo está en el Globo Sempertex Reflex.</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>Marca: Sempertex; Forma: Redondo; Material: Látex natural; Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 85, en 8 familias: Fashion, Pastel Mate, Neón, Pastel Dusk, Satín, Silk, Metálico y Reflex</t>
+          <t>Marca: Sempertex; Forma: Redondo; Material: Látex natural; Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 74, en 7 familias: Fashion, Pastel Mate, Neón, Pastel Dusk, Satín, Silk y Metálico</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>Carta Sempertex</t>
+          <t>Sempertex Fashion, Sempertex Pastel Mate, Sempertex Neón, Sempertex Pastel Dusk, Sempertex Satín, Sempertex Silk, Sempertex Metálico</t>
         </is>
       </c>
       <c r="M21" s="3" t="n"/>
@@ -3139,12 +3139,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-12-estandar-50</t>
+          <t>globo-sempertex-reflex-redondo</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex 12" estándar, bolsa 50 pzas</t>
+          <t>Globo Sempertex Reflex redondo</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -3154,17 +3154,17 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Fiestas infantiles, Baby shower, Revelación de género, Fiestas patrias, Graduación</t>
+          <t>Cumpleaños, Bodas y aniversarios, XV años, Graduación, Navidad</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>85</v>
+        <v>124</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>72</v>
+        <v>99</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
@@ -3172,21 +3172,21 @@
         </is>
       </c>
       <c r="I22" s="3" t="n">
-        <v>160</v>
+        <v>60</v>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Globo redondo de 12 pulgadas en color sólido, de látex natural. Es el más usado para arcos, columnas y decoración con aire o helio. Cada bolsa trae 50 piezas del mismo color.</t>
+          <t>Globo Sempertex Reflex con efecto espejo, tipo cromo. Brilla como metal y luce en arcos, columnas y decoraciones de lujo. El 18" viene en bolsa de 15 o de 25 piezas.</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas; Material: Látex natural biodegradable; Duración con helio: 8 a 12 horas (más con sellador)</t>
+          <t>Marca: Sempertex; Forma: Redondo; Acabado: Reflex (efecto espejo); Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 11 tonos Reflex</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>Rojo, Rosa, Fucsia, Lila, Morado, Azul rey, Azul cielo, Verde limón, Amarillo, Naranja, Blanco, Negro</t>
+          <t>Sempertex Reflex</t>
         </is>
       </c>
       <c r="M22" s="3" t="n"/>
@@ -3195,14 +3195,14 @@
       <c r="P22" s="3" t="n"/>
       <c r="Q22" s="3" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="R22" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="S22" s="3" t="inlineStr">
         <is>
           <t>Visible</t>
@@ -3210,21 +3210,25 @@
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>latex r12 12 pulgadas bolsa colores arco columna</t>
-        </is>
-      </c>
-      <c r="U22" s="3" t="n"/>
+          <t>sempertex reflex cromo espejo metalico latex redondo r5 r12 r18</t>
+        </is>
+      </c>
+      <c r="U22" s="3" t="inlineStr">
+        <is>
+          <t>5"</t>
+        </is>
+      </c>
       <c r="V22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-12-pastel-50</t>
+          <t>globo-sempertex-reflex-redondo</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex 12" pastel, bolsa 50 pzas</t>
+          <t>Globo Sempertex Reflex redondo</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -3234,17 +3238,17 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Baby shower, Revelación de género, XV años, Bodas y aniversarios, Fiestas infantiles</t>
+          <t>Cumpleaños, Bodas y aniversarios, XV años, Graduación, Navidad</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>95</v>
+        <v>314</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>80</v>
+        <v>251.21</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
@@ -3252,21 +3256,21 @@
         </is>
       </c>
       <c r="I23" s="3" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Tonos pastel tipo macaron para decoraciones suaves: baby shower, bautizos y mesas de postres.</t>
+          <t>Globo Sempertex Reflex con efecto espejo, tipo cromo. Brilla como metal y luce en arcos, columnas y decoraciones de lujo. El 18" viene en bolsa de 15 o de 25 piezas.</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
         <is>
-          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas; Acabado: Pastel mate</t>
+          <t>Marca: Sempertex; Forma: Redondo; Acabado: Reflex (efecto espejo); Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 11 tonos Reflex</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>Rosa pastel, Lila pastel, Azul pastel, Menta, Amarillo pastel, Durazno</t>
+          <t>Sempertex Reflex</t>
         </is>
       </c>
       <c r="M23" s="3" t="n"/>
@@ -3290,21 +3294,25 @@
       </c>
       <c r="T23" s="3" t="inlineStr">
         <is>
-          <t>latex pastel macaron baby bautizo</t>
-        </is>
-      </c>
-      <c r="U23" s="3" t="n"/>
+          <t>sempertex reflex cromo espejo metalico latex redondo r5 r12 r18</t>
+        </is>
+      </c>
+      <c r="U23" s="3" t="inlineStr">
+        <is>
+          <t>12"</t>
+        </is>
+      </c>
       <c r="V23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-12-metalico-50</t>
+          <t>globo-sempertex-reflex-redondo</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex 12" metálico perlado, bolsa 50 pzas</t>
+          <t>Globo Sempertex Reflex redondo</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -3314,39 +3322,39 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Bodas y aniversarios, XV años, Graduación, Navidad, Cumpleaños</t>
+          <t>Cumpleaños, Bodas y aniversarios, XV años, Graduación, Navidad</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>110</v>
+        <v>398</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>95</v>
+        <v>318</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>bolsa con 50 piezas</t>
+          <t>bolsa con 15 piezas</t>
         </is>
       </c>
       <c r="I24" s="3" t="n">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Acabado perlado con brillo suave. Combina muy bien con globos foil y decoraciones elegantes.</t>
+          <t>Globo Sempertex Reflex con efecto espejo, tipo cromo. Brilla como metal y luce en arcos, columnas y decoraciones de lujo. El 18" viene en bolsa de 15 o de 25 piezas.</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas; Acabado: Metálico perlado</t>
+          <t>Marca: Sempertex; Forma: Redondo; Acabado: Reflex (efecto espejo); Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 11 tonos Reflex</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>Dorado, Plateado, Oro rosa, Azul, Rojo, Rosa, Morado, Verde</t>
+          <t>Sempertex Reflex</t>
         </is>
       </c>
       <c r="M24" s="3" t="n"/>
@@ -3355,14 +3363,14 @@
       <c r="P24" s="3" t="n"/>
       <c r="Q24" s="3" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="R24" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="S24" s="3" t="inlineStr">
         <is>
           <t>Visible</t>
@@ -3370,21 +3378,25 @@
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>latex metalico perlado brillo</t>
-        </is>
-      </c>
-      <c r="U24" s="3" t="n"/>
+          <t>sempertex reflex cromo espejo metalico latex redondo r5 r12 r18</t>
+        </is>
+      </c>
+      <c r="U24" s="3" t="inlineStr">
+        <is>
+          <t>18" (15 pz)</t>
+        </is>
+      </c>
       <c r="V24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-12-cromado-25</t>
+          <t>globo-sempertex-reflex-redondo</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex cromado 12", bolsa 25 pzas</t>
+          <t>Globo Sempertex Reflex redondo</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -3394,17 +3406,17 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Bodas y aniversarios, XV años, Graduación, Navidad</t>
+          <t>Cumpleaños, Bodas y aniversarios, XV años, Graduación, Navidad</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>120</v>
+        <v>687</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>105</v>
+        <v>550</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
@@ -3412,21 +3424,21 @@
         </is>
       </c>
       <c r="I25" s="3" t="n">
-        <v>85</v>
+        <v>240</v>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Efecto espejo, parecido al foil pero en látex. Para decoraciones de lujo y arcos de evento.</t>
+          <t>Globo Sempertex Reflex con efecto espejo, tipo cromo. Brilla como metal y luce en arcos, columnas y decoraciones de lujo. El 18" viene en bolsa de 15 o de 25 piezas.</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>Medida: 12 in (30 cm) inflado; Contenido: 25 piezas; Acabado: Cromado tipo espejo</t>
+          <t>Marca: Sempertex; Forma: Redondo; Acabado: Reflex (efecto espejo); Tamaños: 5" (13 cm), 12" (30 cm) y 18" (46 cm); Tonos: 11 tonos Reflex</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>Oro cromo #c9a227, Plata cromo #a9b1bb, Oro rosa cromo #d9897a, Champagne cromo #d8c08f, Azul cromo #3767c9</t>
+          <t>Sempertex Reflex</t>
         </is>
       </c>
       <c r="M25" s="3" t="n"/>
@@ -3440,7 +3452,7 @@
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="S25" s="3" t="inlineStr">
@@ -3450,21 +3462,25 @@
       </c>
       <c r="T25" s="3" t="inlineStr">
         <is>
-          <t>latex cromado cromo espejo lujo</t>
-        </is>
-      </c>
-      <c r="U25" s="3" t="n"/>
+          <t>sempertex reflex cromo espejo metalico latex redondo r5 r12 r18</t>
+        </is>
+      </c>
+      <c r="U25" s="3" t="inlineStr">
+        <is>
+          <t>18" (25 pz)</t>
+        </is>
+      </c>
       <c r="V25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-5-mini-100</t>
+          <t>globo-latex-12-estandar-50</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex 5" mini, bolsa 100 pzas</t>
+          <t>Globo de látex 12" estándar, bolsa 50 pzas</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -3474,39 +3490,39 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Baby shower, Cumpleaños, Bodas y aniversarios</t>
+          <t>Cumpleaños, Fiestas infantiles, Baby shower, Revelación de género, Fiestas patrias, Graduación</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>6</v>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>bolsa con 100 piezas</t>
+          <t>bolsa con 50 piezas</t>
         </is>
       </c>
       <c r="I26" s="3" t="n">
-        <v>110</v>
+        <v>160</v>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Globito de 5 pulgadas para dar textura a arcos orgánicos, rellenar burbujas y decorar mesas.</t>
+          <t>Globo redondo de 12 pulgadas en color sólido, de látex natural. Es el más usado para arcos, columnas y decoración con aire o helio. Cada bolsa trae 50 piezas del mismo color.</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>Medida: 5 in (13 cm) inflado; Contenido: 100 piezas; Material: Látex natural</t>
+          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas; Material: Látex natural biodegradable; Duración con helio: 8 a 12 horas (más con sellador)</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>Rosa, Rojo, Azul rey, Verde limón, Lila, Amarillo, Blanco, Negro</t>
+          <t>Rojo, Rosa, Fucsia, Lila, Morado, Azul rey, Azul cielo, Verde limón, Amarillo, Naranja, Blanco, Negro</t>
         </is>
       </c>
       <c r="M26" s="3" t="n"/>
@@ -3515,14 +3531,14 @@
       <c r="P26" s="3" t="n"/>
       <c r="Q26" s="3" t="inlineStr">
         <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="R26" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="S26" s="3" t="inlineStr">
         <is>
           <t>Visible</t>
@@ -3530,7 +3546,7 @@
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>latex mini 5 pulgadas chico arco organico relleno</t>
+          <t>latex r12 12 pulgadas bolsa colores arco columna</t>
         </is>
       </c>
       <c r="U26" s="3" t="n"/>
@@ -3539,12 +3555,12 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-18-10</t>
+          <t>globo-latex-12-pastel-50</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex 18", bolsa 10 pzas</t>
+          <t>Globo de látex 12" pastel, bolsa 50 pzas</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -3554,39 +3570,39 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Baby shower, Bodas y aniversarios</t>
+          <t>Baby shower, Revelación de género, XV años, Bodas y aniversarios, Fiestas infantiles</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>6</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>bolsa con 10 piezas</t>
+          <t>bolsa con 50 piezas</t>
         </is>
       </c>
       <c r="I27" s="3" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Globo grande de 18 pulgadas para dar volumen en arcos y columnas.</t>
+          <t>Tonos pastel tipo macaron para decoraciones suaves: baby shower, bautizos y mesas de postres.</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
         <is>
-          <t>Medida: 18 in (45 cm) inflado; Contenido: 10 piezas; Material: Látex natural</t>
+          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas; Acabado: Pastel mate</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>Azul cielo, Rosa, Rojo, Amarillo, Blanco, Negro</t>
+          <t>Rosa pastel, Lila pastel, Azul pastel, Menta, Amarillo pastel, Durazno</t>
         </is>
       </c>
       <c r="M27" s="3" t="n"/>
@@ -3600,7 +3616,7 @@
       </c>
       <c r="R27" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="S27" s="3" t="inlineStr">
@@ -3610,7 +3626,7 @@
       </c>
       <c r="T27" s="3" t="inlineStr">
         <is>
-          <t>latex 18 pulgadas grande arco columna</t>
+          <t>latex pastel macaron baby bautizo</t>
         </is>
       </c>
       <c r="U27" s="3" t="n"/>
@@ -3619,12 +3635,12 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-260-50</t>
+          <t>globo-latex-12-metalico-50</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex 260 para figuras, bolsa 50 pzas</t>
+          <t>Globo de látex 12" metálico perlado, bolsa 50 pzas</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -3634,14 +3650,14 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Fiestas infantiles, Cumpleaños</t>
+          <t>Bodas y aniversarios, XV años, Graduación, Navidad, Cumpleaños</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="G28" s="3" t="n">
         <v>6</v>
@@ -3652,21 +3668,21 @@
         </is>
       </c>
       <c r="I28" s="3" t="n">
-        <v>150</v>
+        <v>165</v>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>Globo largo para hacer perritos, espadas, flores y figuras. Se infla con inflador manual.</t>
+          <t>Acabado perlado con brillo suave. Combina muy bien con globos foil y decoraciones elegantes.</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>Medida: 5 × 150 cm inflado (260Q); Contenido: 50 piezas; Inflado: Con inflador manual</t>
+          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas; Acabado: Metálico perlado</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>Surtido, Blanco, Rojo, Azul, Verde, Amarillo, Negro</t>
+          <t>Dorado, Plateado, Oro rosa, Azul, Rojo, Rosa, Morado, Verde</t>
         </is>
       </c>
       <c r="M28" s="3" t="n"/>
@@ -3675,14 +3691,14 @@
       <c r="P28" s="3" t="n"/>
       <c r="Q28" s="3" t="inlineStr">
         <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="R28" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="S28" s="3" t="inlineStr">
         <is>
           <t>Visible</t>
@@ -3690,7 +3706,7 @@
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>latex 260 largo figuras perrito payaso globoflexia</t>
+          <t>latex metalico perlado brillo</t>
         </is>
       </c>
       <c r="U28" s="3" t="n"/>
@@ -3699,12 +3715,12 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-confeti-12-10</t>
+          <t>globo-latex-12-cromado-25</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Globo transparente con confeti 12", bolsa 10 pzas</t>
+          <t>Globo de látex cromado 12", bolsa 25 pzas</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -3714,39 +3730,39 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Bodas y aniversarios, XV años, Baby shower</t>
+          <t>Bodas y aniversarios, XV años, Graduación, Navidad</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>55</v>
+        <v>105</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>6</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>bolsa con 10 piezas</t>
+          <t>bolsa con 25 piezas</t>
         </is>
       </c>
       <c r="I29" s="3" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Globo transparente que ya trae confeti metálico dentro. Al inflarlo y frotarlo, el confeti se pega a las paredes.</t>
+          <t>Efecto espejo, parecido al foil pero en látex. Para decoraciones de lujo y arcos de evento.</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>Medida: 12 in (30 cm) inflado; Contenido: 10 globos con confeti incluido</t>
+          <t>Medida: 12 in (30 cm) inflado; Contenido: 25 piezas; Acabado: Cromado tipo espejo</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>Dorado, Plateado, Oro rosa, Rosa, Azul</t>
+          <t>Oro cromo #c9a227, Plata cromo #a9b1bb, Oro rosa cromo #d9897a, Champagne cromo #d8c08f, Azul cromo #3767c9</t>
         </is>
       </c>
       <c r="M29" s="3" t="n"/>
@@ -3760,7 +3776,7 @@
       </c>
       <c r="R29" s="3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="S29" s="3" t="inlineStr">
@@ -3770,7 +3786,7 @@
       </c>
       <c r="T29" s="3" t="inlineStr">
         <is>
-          <t>latex confeti transparente brillos</t>
+          <t>latex cromado cromo espejo lujo</t>
         </is>
       </c>
       <c r="U29" s="3" t="n"/>
@@ -3779,12 +3795,12 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-corazon-12-50</t>
+          <t>globo-latex-5-mini-100</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex corazón 12", bolsa 50 pzas</t>
+          <t>Globo de látex 5" mini, bolsa 100 pzas</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -3794,39 +3810,39 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Amor y amistad, Bodas y aniversarios, XV años</t>
+          <t>Baby shower, Cumpleaños, Bodas y aniversarios</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="G30" s="3" t="n">
         <v>6</v>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>bolsa con 50 piezas</t>
+          <t>bolsa con 100 piezas</t>
         </is>
       </c>
       <c r="I30" s="3" t="n">
-        <v>170</v>
+        <v>110</v>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>Globos de látex en forma de corazón para San Valentín, bodas y declaraciones.</t>
+          <t>Globito de 5 pulgadas para dar textura a arcos orgánicos, rellenar burbujas y decorar mesas.</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas</t>
+          <t>Medida: 5 in (13 cm) inflado; Contenido: 100 piezas; Material: Látex natural</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>Rojo, Rosa, Fucsia, Blanco</t>
+          <t>Rosa, Rojo, Azul rey, Verde limón, Lila, Amarillo, Blanco, Negro</t>
         </is>
       </c>
       <c r="M30" s="3" t="n"/>
@@ -3850,7 +3866,7 @@
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>latex corazon corazones amor san valentin</t>
+          <t>latex mini 5 pulgadas chico arco organico relleno</t>
         </is>
       </c>
       <c r="U30" s="3" t="n"/>
@@ -3859,12 +3875,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-feliz-cumple-12-50</t>
+          <t>globo-latex-18-10</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex impreso "Feliz Cumple", bolsa 50 pzas</t>
+          <t>Globo de látex 18", bolsa 10 pzas</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -3874,37 +3890,41 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Fiestas infantiles</t>
+          <t>Cumpleaños, Baby shower, Bodas y aniversarios</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>110</v>
+        <v>75</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>95</v>
+        <v>64</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>6</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>bolsa con 50 piezas</t>
+          <t>bolsa con 10 piezas</t>
         </is>
       </c>
       <c r="I31" s="3" t="n">
-        <v>165</v>
+        <v>120</v>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Globos de 12 pulgadas en colores surtidos con "Feliz Cumpleaños" impreso alrededor.</t>
+          <t>Globo grande de 18 pulgadas para dar volumen en arcos y columnas.</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas en colores surtidos; Impresión: A una tinta, todo alrededor</t>
-        </is>
-      </c>
-      <c r="L31" s="3" t="n"/>
+          <t>Medida: 18 in (45 cm) inflado; Contenido: 10 piezas; Material: Látex natural</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Azul cielo, Rosa, Rojo, Amarillo, Blanco, Negro</t>
+        </is>
+      </c>
       <c r="M31" s="3" t="n"/>
       <c r="N31" s="3" t="n"/>
       <c r="O31" s="3" t="n"/>
@@ -3926,7 +3946,7 @@
       </c>
       <c r="T31" s="3" t="inlineStr">
         <is>
-          <t>latex impreso feliz cumpleaños cumple surtido</t>
+          <t>latex 18 pulgadas grande arco columna</t>
         </is>
       </c>
       <c r="U31" s="3" t="n"/>
@@ -3935,12 +3955,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>globo-latex-36-gigante</t>
+          <t>globo-latex-260-50</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Globo de látex gigante 36"</t>
+          <t>Globo de látex 260 para figuras, bolsa 50 pzas</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -3950,39 +3970,39 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Baby shower, Revelación de género, Bodas y aniversarios</t>
+          <t>Fiestas infantiles, Cumpleaños</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>pieza</t>
+          <t>bolsa con 50 piezas</t>
         </is>
       </c>
       <c r="I32" s="3" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>Globo de 3 pies (90 cm) para fotos, revelaciones de género y como pieza central de una decoración.</t>
+          <t>Globo largo para hacer perritos, espadas, flores y figuras. Se infla con inflador manual.</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>Medida: 36 in (90 cm) inflado; Material: Látex natural grueso</t>
+          <t>Medida: 5 × 150 cm inflado (260Q); Contenido: 50 piezas; Inflado: Con inflador manual</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>Rosa, Rojo, Azul cielo, Dorado, Blanco, Negro</t>
+          <t>Surtido, Blanco, Rojo, Azul, Verde, Amarillo, Negro</t>
         </is>
       </c>
       <c r="M32" s="3" t="n"/>
@@ -4006,7 +4026,7 @@
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>latex gigante 36 jumbo grande revelacion</t>
+          <t>latex 260 largo figuras perrito payaso globoflexia</t>
         </is>
       </c>
       <c r="U32" s="3" t="n"/>
@@ -4015,12 +4035,12 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>kit-arco-organico</t>
+          <t>globo-latex-confeti-12-10</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Kit arco orgánico de globos (100 pzas)</t>
+          <t>Globo transparente con confeti 12", bolsa 10 pzas</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -4030,59 +4050,55 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Baby shower, Cumpleaños, Bodas y aniversarios, XV años, Revelación de género</t>
+          <t>Cumpleaños, Bodas y aniversarios, XV años, Baby shower</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>260</v>
+        <v>65</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>235</v>
+        <v>55</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>kit</t>
+          <t>bolsa con 10 piezas</t>
         </is>
       </c>
       <c r="I33" s="3" t="n">
-        <v>420</v>
+        <v>70</v>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Todo para armar un arco orgánico de 2.5 a 3 metros: 100 globos en tres tamaños, cinta para arco y puntos de pegamento.</t>
+          <t>Globo transparente que ya trae confeti metálico dentro. Al inflarlo y frotarlo, el confeti se pega a las paredes.</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>Incluye: 100 globos (5", 10" y 12"), 5 m de cinta y 1 rollo de puntos de pegamento; Largo aproximado: 2.5 a 3 m</t>
-        </is>
-      </c>
-      <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Paleta</t>
-        </is>
-      </c>
-      <c r="N33" s="3" t="inlineStr">
-        <is>
-          <t>Rosa y dorado, Azul y plata, Pastel arcoíris, Salvia y blanco, Negro y dorado</t>
-        </is>
-      </c>
+          <t>Medida: 12 in (30 cm) inflado; Contenido: 10 globos con confeti incluido</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Dorado, Plateado, Oro rosa, Rosa, Azul</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="n"/>
+      <c r="N33" s="3" t="n"/>
       <c r="O33" s="3" t="n"/>
       <c r="P33" s="3" t="n"/>
       <c r="Q33" s="3" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="R33" s="3" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
       <c r="S33" s="3" t="inlineStr">
         <is>
           <t>Visible</t>
@@ -4090,7 +4106,7 @@
       </c>
       <c r="T33" s="3" t="inlineStr">
         <is>
-          <t>kit arco organico guirnalda decoracion set</t>
+          <t>latex confeti transparente brillos</t>
         </is>
       </c>
       <c r="U33" s="3" t="n"/>
@@ -4099,12 +4115,12 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>inflador-manual-doble-accion</t>
+          <t>globo-latex-corazon-12-50</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Inflador manual de doble acción</t>
+          <t>Globo de látex corazón 12", bolsa 50 pzas</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -4112,37 +4128,41 @@
           <t>Globos de látex</t>
         </is>
       </c>
-      <c r="D34" s="3" t="n"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Amor y amistad, Bodas y aniversarios, XV años</t>
+        </is>
+      </c>
       <c r="E34" s="4" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="G34" s="3" t="n">
         <v>6</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>pieza</t>
+          <t>bolsa con 50 piezas</t>
         </is>
       </c>
       <c r="I34" s="3" t="n">
-        <v>320</v>
+        <v>170</v>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Infla al subir y al bajar, así terminas el doble de rápido. Sirve para látex, globos 260 y foil con aire.</t>
+          <t>Globos de látex en forma de corazón para San Valentín, bodas y declaraciones.</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>Largo: 30 cm; Uso: Látex, 260 y foil chico; Incluye: Boquilla para globo 260</t>
+          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>Azul, Rosa, Morado</t>
+          <t>Rojo, Rosa, Fucsia, Blanco</t>
         </is>
       </c>
       <c r="M34" s="3" t="n"/>
@@ -4166,7 +4186,7 @@
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>inflador bomba accesorio herramienta</t>
+          <t>latex corazon corazones amor san valentin</t>
         </is>
       </c>
       <c r="U34" s="3" t="n"/>
@@ -4175,12 +4195,12 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>cinta-para-arco-5m</t>
+          <t>globo-latex-feliz-cumple-12-50</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Cinta para arco de globos, 5 m</t>
+          <t>Globo de látex impreso "Feliz Cumple", bolsa 50 pzas</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -4188,32 +4208,36 @@
           <t>Globos de látex</t>
         </is>
       </c>
-      <c r="D35" s="3" t="n"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Cumpleaños, Fiestas infantiles</t>
+        </is>
+      </c>
       <c r="E35" s="4" t="n">
-        <v>25</v>
+        <v>110</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>rollo de 5 m</t>
+          <t>bolsa con 50 piezas</t>
         </is>
       </c>
       <c r="I35" s="3" t="n">
-        <v>35</v>
+        <v>165</v>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>Tira de plástico con orificios para insertar los nudos de los globos y armar arcos y guirnaldas sin pegamento.</t>
+          <t>Globos de 12 pulgadas en colores surtidos con "Feliz Cumpleaños" impreso alrededor.</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>Largo: 5 m; Material: PVC transparente</t>
+          <t>Medida: 12 in (30 cm) inflado; Contenido: 50 piezas en colores surtidos; Impresión: A una tinta, todo alrededor</t>
         </is>
       </c>
       <c r="L35" s="3" t="n"/>
@@ -4238,7 +4262,7 @@
       </c>
       <c r="T35" s="3" t="inlineStr">
         <is>
-          <t>cinta arco tira accesorio guirnalda</t>
+          <t>latex impreso feliz cumpleaños cumple surtido</t>
         </is>
       </c>
       <c r="U35" s="3" t="n"/>
@@ -4247,54 +4271,54 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>papel-china-50-pliegos</t>
+          <t>globo-latex-36-gigante</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Papel china, paquete 50 pliegos</t>
+          <t>Globo de látex gigante 36"</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Papelería</t>
+          <t>Globos de látex</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Fiestas patrias, Navidad, Cumpleaños, Fiestas infantiles</t>
+          <t>Cumpleaños, Baby shower, Revelación de género, Bodas y aniversarios</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>paquete con 50 pliegos</t>
+          <t>pieza</t>
         </is>
       </c>
       <c r="I36" s="3" t="n">
-        <v>330</v>
+        <v>30</v>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>Papel de china para piñatas, papel picado, flores, borlas y manualidades. Paquete de 50 pliegos de un solo color.</t>
+          <t>Globo de 3 pies (90 cm) para fotos, revelaciones de género y como pieza central de una decoración.</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>Medida del pliego: 50 × 75 cm; Contenido: 50 pliegos</t>
+          <t>Medida: 36 in (90 cm) inflado; Material: Látex natural grueso</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>Rosa, Fucsia, Rojo, Naranja, Amarillo, Verde bandera, Verde limón, Azul cielo, Azul rey, Morado, Blanco, Negro</t>
+          <t>Rosa, Rojo, Azul cielo, Dorado, Blanco, Negro</t>
         </is>
       </c>
       <c r="M36" s="3" t="n"/>
@@ -4303,7 +4327,7 @@
       <c r="P36" s="3" t="n"/>
       <c r="Q36" s="3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="R36" s="3" t="inlineStr">
@@ -4318,7 +4342,7 @@
       </c>
       <c r="T36" s="3" t="inlineStr">
         <is>
-          <t>papel china piñata manualidades pliegos</t>
+          <t>latex gigante 36 jumbo grande revelacion</t>
         </is>
       </c>
       <c r="U36" s="3" t="n"/>
@@ -4327,68 +4351,72 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>papel-crepe-pliego</t>
+          <t>kit-arco-organico</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Papel crepé, pliego 50 × 200 cm</t>
+          <t>Kit arco orgánico de globos (100 pzas)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Papelería</t>
+          <t>Globos de látex</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Fiestas infantiles, Fiestas patrias, Navidad</t>
+          <t>Baby shower, Cumpleaños, Bodas y aniversarios, XV años, Revelación de género</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>9</v>
+        <v>260</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>7</v>
+        <v>235</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>pliego</t>
+          <t>kit</t>
         </is>
       </c>
       <c r="I37" s="3" t="n">
-        <v>35</v>
+        <v>420</v>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>Papel crepé elástico para flores, disfraces, cortinas y forrar mesas.</t>
+          <t>Todo para armar un arco orgánico de 2.5 a 3 metros: 100 globos en tres tamaños, cinta para arco y puntos de pegamento.</t>
         </is>
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>Medida: 50 × 200 cm; Textura: Corrugado elástico</t>
-        </is>
-      </c>
-      <c r="L37" s="3" t="inlineStr">
-        <is>
-          <t>Rojo, Rosa, Amarillo, Verde, Azul, Morado, Naranja, Blanco, Negro</t>
-        </is>
-      </c>
-      <c r="M37" s="3" t="n"/>
-      <c r="N37" s="3" t="n"/>
+          <t>Incluye: 100 globos (5", 10" y 12"), 5 m de cinta y 1 rollo de puntos de pegamento; Largo aproximado: 2.5 a 3 m</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="n"/>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>Paleta</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>Rosa y dorado, Azul y plata, Pastel arcoíris, Salvia y blanco, Negro y dorado</t>
+        </is>
+      </c>
       <c r="O37" s="3" t="n"/>
       <c r="P37" s="3" t="n"/>
       <c r="Q37" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="R37" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="S37" s="3" t="inlineStr">
@@ -4398,7 +4426,7 @@
       </c>
       <c r="T37" s="3" t="inlineStr">
         <is>
-          <t>papel crepe crepé flores disfraz manualidades</t>
+          <t>kit arco organico guirnalda decoracion set</t>
         </is>
       </c>
       <c r="U37" s="3" t="n"/>
@@ -4407,50 +4435,50 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>cartulina-pliego</t>
+          <t>inflador-manual-doble-accion</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Cartulina, pliego 50 × 65 cm</t>
+          <t>Inflador manual de doble acción</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Papelería</t>
+          <t>Globos de látex</t>
         </is>
       </c>
       <c r="D38" s="3" t="n"/>
       <c r="E38" s="4" t="n">
-        <v>8</v>
+        <v>85</v>
       </c>
       <c r="F38" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="G38" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="G38" s="3" t="n">
-        <v>25</v>
-      </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>pliego</t>
+          <t>pieza</t>
         </is>
       </c>
       <c r="I38" s="3" t="n">
-        <v>65</v>
+        <v>320</v>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Cartulina de colores para letreros, carteles, tareas y manualidades.</t>
+          <t>Infla al subir y al bajar, así terminas el doble de rápido. Sirve para látex, globos 260 y foil con aire.</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>Medida: 50 × 65 cm; Gramaje: 180 g/m² aprox.</t>
+          <t>Largo: 30 cm; Uso: Látex, 260 y foil chico; Incluye: Boquilla para globo 260</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
         <is>
-          <t>Amarillo, Rosa, Rojo, Verde, Azul cielo, Azul rey, Naranja, Morado, Blanco, Negro</t>
+          <t>Azul, Rosa, Morado</t>
         </is>
       </c>
       <c r="M38" s="3" t="n"/>
@@ -4474,7 +4502,7 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>cartulina carteles letrero escolar</t>
+          <t>inflador bomba accesorio herramienta</t>
         </is>
       </c>
       <c r="U38" s="3" t="n"/>
@@ -4483,67 +4511,55 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>papel-picado-plastico-5m</t>
+          <t>cinta-para-arco-5m</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Papel picado de plástico, tira 5 m</t>
+          <t>Cinta para arco de globos, 5 m</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Papelería</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Navidad, Fiestas patrias, Bodas y aniversarios, XV años, Cumpleaños</t>
-        </is>
-      </c>
+          <t>Globos de látex</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n"/>
       <c r="E39" s="4" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>tira de 5 m</t>
+          <t>rollo de 5 m</t>
         </is>
       </c>
       <c r="I39" s="3" t="n">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>Papel picado de plástico resistente al aire y la lluvia, para posadas, patios y salones. Tira de 5 metros con 10 pliegos.</t>
+          <t>Tira de plástico con orificios para insertar los nudos de los globos y armar arcos y guirnaldas sin pegamento.</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>Largo: 5 m con 10 pliegos; Material: Plástico, se puede reusar</t>
+          <t>Largo: 5 m; Material: PVC transparente</t>
         </is>
       </c>
       <c r="L39" s="3" t="n"/>
-      <c r="M39" s="3" t="inlineStr">
-        <is>
-          <t>Diseño</t>
-        </is>
-      </c>
-      <c r="N39" s="3" t="inlineStr">
-        <is>
-          <t>Multicolor, Navidad, Tricolor, Blanco y dorado</t>
-        </is>
-      </c>
+      <c r="M39" s="3" t="n"/>
+      <c r="N39" s="3" t="n"/>
       <c r="O39" s="3" t="n"/>
       <c r="P39" s="3" t="n"/>
       <c r="Q39" s="3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="R39" s="3" t="inlineStr">
@@ -4558,7 +4574,7 @@
       </c>
       <c r="T39" s="3" t="inlineStr">
         <is>
-          <t>papel picado plastico posada navidad fiestas patrias</t>
+          <t>cinta arco tira accesorio guirnalda</t>
         </is>
       </c>
       <c r="U39" s="3" t="n"/>
@@ -4567,12 +4583,12 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>banderin-feliz-cumpleanos</t>
+          <t>papel-china-50-pliegos</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Banderín "Feliz Cumpleaños", 2.5 m</t>
+          <t>Papel china, paquete 50 pliegos</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -4582,59 +4598,55 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Fiestas infantiles</t>
+          <t>Fiestas patrias, Navidad, Cumpleaños, Fiestas infantiles</t>
         </is>
       </c>
       <c r="E40" s="4" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>pieza</t>
+          <t>paquete con 50 pliegos</t>
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>60</v>
+        <v>330</v>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>Guirnalda de banderines con la frase "Feliz Cumpleaños", ya armada con cordón.</t>
+          <t>Papel de china para piñatas, papel picado, flores, borlas y manualidades. Paquete de 50 pliegos de un solo color.</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t>Largo: 2.5 m; Material: Cartulina gruesa</t>
-        </is>
-      </c>
-      <c r="L40" s="3" t="n"/>
-      <c r="M40" s="3" t="inlineStr">
-        <is>
-          <t>Color</t>
-        </is>
-      </c>
-      <c r="N40" s="3" t="inlineStr">
-        <is>
-          <t>Dorado, Multicolor, Rosa, Azul</t>
-        </is>
-      </c>
+          <t>Medida del pliego: 50 × 75 cm; Contenido: 50 pliegos</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Rosa, Fucsia, Rojo, Naranja, Amarillo, Verde bandera, Verde limón, Azul cielo, Azul rey, Morado, Blanco, Negro</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="n"/>
+      <c r="N40" s="3" t="n"/>
       <c r="O40" s="3" t="n"/>
       <c r="P40" s="3" t="n"/>
       <c r="Q40" s="3" t="inlineStr">
         <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R40" s="3" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="R40" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="S40" s="3" t="inlineStr">
         <is>
           <t>Visible</t>
@@ -4642,7 +4654,7 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>banderin guirnalda letrero feliz cumpleaños</t>
+          <t>papel china piñata manualidades pliegos</t>
         </is>
       </c>
       <c r="U40" s="3" t="n"/>
@@ -4651,12 +4663,12 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>invitaciones-paquete-10</t>
+          <t>papel-crepe-pliego</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Invitaciones con sobre, paquete 10</t>
+          <t>Papel crepé, pliego 50 × 200 cm</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -4666,47 +4678,43 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Fiestas infantiles, Baby shower, XV años, Bodas y aniversarios</t>
+          <t>Fiestas infantiles, Fiestas patrias, Navidad</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>paquete con 10 invitaciones</t>
+          <t>pliego</t>
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>Invitaciones impresas para llenar a mano, con sobre. Elige el diseño de tu evento.</t>
+          <t>Papel crepé elástico para flores, disfraces, cortinas y forrar mesas.</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>Medida: 10 × 15 cm; Contenido: 10 invitaciones y 10 sobres</t>
-        </is>
-      </c>
-      <c r="L41" s="3" t="n"/>
-      <c r="M41" s="3" t="inlineStr">
-        <is>
-          <t>Diseño</t>
-        </is>
-      </c>
-      <c r="N41" s="3" t="inlineStr">
-        <is>
-          <t>Cumpleaños infantil, Baby shower, XV años, Boda</t>
-        </is>
-      </c>
+          <t>Medida: 50 × 200 cm; Textura: Corrugado elástico</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Rojo, Rosa, Amarillo, Verde, Azul, Morado, Naranja, Blanco, Negro</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="n"/>
+      <c r="N41" s="3" t="n"/>
       <c r="O41" s="3" t="n"/>
       <c r="P41" s="3" t="n"/>
       <c r="Q41" s="3" t="inlineStr">
@@ -4726,7 +4734,7 @@
       </c>
       <c r="T41" s="3" t="inlineStr">
         <is>
-          <t>invitaciones invitacion sobre tarjetas</t>
+          <t>papel crepe crepé flores disfraz manualidades</t>
         </is>
       </c>
       <c r="U41" s="3" t="n"/>
@@ -4735,12 +4743,12 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>foami-carta-10</t>
+          <t>cartulina-pliego</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Foami tamaño carta, paquete 10 hojas</t>
+          <t>Cartulina, pliego 50 × 65 cm</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -4748,41 +4756,37 @@
           <t>Papelería</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>Fiestas infantiles</t>
-        </is>
-      </c>
+      <c r="D42" s="3" t="n"/>
       <c r="E42" s="4" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>paquete con 10 hojas</t>
+          <t>pliego</t>
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>110</v>
+        <v>65</v>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>Hojas de foami de 2 mm para manualidades, letreros y decoración escolar.</t>
+          <t>Cartulina de colores para letreros, carteles, tareas y manualidades.</t>
         </is>
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>Medida: Carta (21.5 × 28 cm); Grosor: 2 mm; Contenido: 10 hojas</t>
+          <t>Medida: 50 × 65 cm; Gramaje: 180 g/m² aprox.</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>Rojo, Rosa, Amarillo, Verde, Azul, Morado, Naranja, Blanco, Negro, Café</t>
+          <t>Amarillo, Rosa, Rojo, Verde, Azul cielo, Azul rey, Naranja, Morado, Blanco, Negro</t>
         </is>
       </c>
       <c r="M42" s="3" t="n"/>
@@ -4806,7 +4810,7 @@
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>foami fomi goma eva manualidades escolar</t>
+          <t>cartulina carteles letrero escolar</t>
         </is>
       </c>
       <c r="U42" s="3" t="n"/>
@@ -4815,12 +4819,12 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>foami-diamantado-carta-5</t>
+          <t>papel-picado-plastico-5m</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Foami diamantado carta, paquete 5 hojas</t>
+          <t>Papel picado de plástico, tira 5 m</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -4830,55 +4834,59 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>XV años, Navidad, Fiestas infantiles</t>
+          <t>Navidad, Fiestas patrias, Bodas y aniversarios, XV años, Cumpleaños</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="G43" s="3" t="n">
         <v>10</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>paquete con 5 hojas</t>
+          <t>tira de 5 m</t>
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>Foami con brillantina que no se cae. Para coronas, letreros y adornos con brillo.</t>
+          <t>Papel picado de plástico resistente al aire y la lluvia, para posadas, patios y salones. Tira de 5 metros con 10 pliegos.</t>
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t>Medida: Carta (21.5 × 28 cm); Contenido: 5 hojas</t>
-        </is>
-      </c>
-      <c r="L43" s="3" t="inlineStr">
-        <is>
-          <t>Dorado, Plateado, Rosa, Rojo, Azul, Morado, Verde</t>
-        </is>
-      </c>
-      <c r="M43" s="3" t="n"/>
-      <c r="N43" s="3" t="n"/>
+          <t>Largo: 5 m con 10 pliegos; Material: Plástico, se puede reusar</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="n"/>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr">
+        <is>
+          <t>Multicolor, Navidad, Tricolor, Blanco y dorado</t>
+        </is>
+      </c>
       <c r="O43" s="3" t="n"/>
       <c r="P43" s="3" t="n"/>
       <c r="Q43" s="3" t="inlineStr">
         <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R43" s="3" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="R43" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="S43" s="3" t="inlineStr">
         <is>
           <t>Visible</t>
@@ -4886,7 +4894,7 @@
       </c>
       <c r="T43" s="3" t="inlineStr">
         <is>
-          <t>foami diamantado brillantina glitter escarchado</t>
+          <t>papel picado plastico posada navidad fiestas patrias</t>
         </is>
       </c>
       <c r="U43" s="3" t="n"/>
@@ -4895,12 +4903,12 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>papel-metalico-pliego</t>
+          <t>banderin-feliz-cumpleanos</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Papel metálico, pliego 50 × 70 cm</t>
+          <t>Banderín "Feliz Cumpleaños", 2.5 m</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -4910,43 +4918,47 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Navidad, Graduación</t>
+          <t>Cumpleaños, Fiestas infantiles</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>pliego</t>
+          <t>pieza</t>
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>Papel con acabado espejo para forrar cajas, hacer moños y decorar fondos.</t>
+          <t>Guirnalda de banderines con la frase "Feliz Cumpleaños", ya armada con cordón.</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>Medida: 50 × 70 cm; Acabado: Metálico brillante</t>
-        </is>
-      </c>
-      <c r="L44" s="3" t="inlineStr">
-        <is>
-          <t>Dorado, Plateado, Rojo, Verde, Azul, Rosa</t>
-        </is>
-      </c>
-      <c r="M44" s="3" t="n"/>
-      <c r="N44" s="3" t="n"/>
+          <t>Largo: 2.5 m; Material: Cartulina gruesa</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="n"/>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="N44" s="3" t="inlineStr">
+        <is>
+          <t>Dorado, Multicolor, Rosa, Azul</t>
+        </is>
+      </c>
       <c r="O44" s="3" t="n"/>
       <c r="P44" s="3" t="n"/>
       <c r="Q44" s="3" t="inlineStr">
@@ -4966,7 +4978,7 @@
       </c>
       <c r="T44" s="3" t="inlineStr">
         <is>
-          <t>papel metalico espejo lustre brillante</t>
+          <t>banderin guirnalda letrero feliz cumpleaños</t>
         </is>
       </c>
       <c r="U44" s="3" t="n"/>
@@ -4975,12 +4987,12 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>topper-feliz-cumple</t>
+          <t>invitaciones-paquete-10</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Topper para pastel "Feliz Cumple"</t>
+          <t>Invitaciones con sobre, paquete 10</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -4990,43 +5002,47 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños</t>
+          <t>Cumpleaños, Fiestas infantiles, Baby shower, XV años, Bodas y aniversarios</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>pieza</t>
+          <t>paquete con 10 invitaciones</t>
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>Adorno para pastel de cartulina metálica, con palitos para insertar.</t>
+          <t>Invitaciones impresas para llenar a mano, con sobre. Elige el diseño de tu evento.</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>Medida: 15 × 12 cm; Material: Cartulina metálica</t>
-        </is>
-      </c>
-      <c r="L45" s="3" t="inlineStr">
-        <is>
-          <t>Dorado, Plateado, Oro rosa, Negro</t>
-        </is>
-      </c>
-      <c r="M45" s="3" t="n"/>
-      <c r="N45" s="3" t="n"/>
+          <t>Medida: 10 × 15 cm; Contenido: 10 invitaciones y 10 sobres</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="n"/>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="inlineStr">
+        <is>
+          <t>Cumpleaños infantil, Baby shower, XV años, Boda</t>
+        </is>
+      </c>
       <c r="O45" s="3" t="n"/>
       <c r="P45" s="3" t="n"/>
       <c r="Q45" s="3" t="inlineStr">
@@ -5046,7 +5062,7 @@
       </c>
       <c r="T45" s="3" t="inlineStr">
         <is>
-          <t>topper pastel adorno cake</t>
+          <t>invitaciones invitacion sobre tarjetas</t>
         </is>
       </c>
       <c r="U45" s="3" t="n"/>
@@ -5055,67 +5071,63 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>papel-envolver-rollo-5m</t>
+          <t>foami-carta-10</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Papel para envolver, rollo 70 cm × 5 m</t>
+          <t>Foami tamaño carta, paquete 10 hojas</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Envolturas</t>
+          <t>Papelería</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Fiestas infantiles, Baby shower, Navidad, Amor y amistad, Bodas y aniversarios</t>
+          <t>Fiestas infantiles</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G46" s="3" t="n">
         <v>10</v>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>rollo</t>
+          <t>paquete con 10 hojas</t>
         </is>
       </c>
       <c r="I46" s="3" t="n">
-        <v>260</v>
+        <v>110</v>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>Papel para regalo en rollo con tubo de cartón. Alcanza para envolver de 8 a 10 regalos medianos.</t>
+          <t>Hojas de foami de 2 mm para manualidades, letreros y decoración escolar.</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>Medida: 70 cm × 5 m; Papel: Couché 60 g/m²</t>
-        </is>
-      </c>
-      <c r="L46" s="3" t="n"/>
-      <c r="M46" s="3" t="inlineStr">
-        <is>
-          <t>Diseño</t>
-        </is>
-      </c>
-      <c r="N46" s="3" t="inlineStr">
-        <is>
-          <t>Cumpleaños, Infantil, Baby, Elegante negro y dorado, Navidad, Amor</t>
-        </is>
-      </c>
+          <t>Medida: Carta (21.5 × 28 cm); Grosor: 2 mm; Contenido: 10 hojas</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>Rojo, Rosa, Amarillo, Verde, Azul, Morado, Naranja, Blanco, Negro, Café</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="n"/>
+      <c r="N46" s="3" t="n"/>
       <c r="O46" s="3" t="n"/>
       <c r="P46" s="3" t="n"/>
       <c r="Q46" s="3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="R46" s="3" t="inlineStr">
@@ -5130,7 +5142,7 @@
       </c>
       <c r="T46" s="3" t="inlineStr">
         <is>
-          <t>papel envolver regalo rollo envoltura</t>
+          <t>foami fomi goma eva manualidades escolar</t>
         </is>
       </c>
       <c r="U46" s="3" t="n"/>
@@ -5139,62 +5151,58 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>papel-envolver-pliegos-25</t>
+          <t>foami-diamantado-carta-5</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Papel para envolver, paquete 25 pliegos</t>
+          <t>Foami diamantado carta, paquete 5 hojas</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Envolturas</t>
+          <t>Papelería</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Fiestas infantiles, Baby shower, Navidad, Amor y amistad, Bodas y aniversarios</t>
+          <t>XV años, Navidad, Fiestas infantiles</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>105</v>
+        <v>33</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>paquete con 25 pliegos</t>
+          <t>paquete con 5 hojas</t>
         </is>
       </c>
       <c r="I47" s="3" t="n">
-        <v>950</v>
+        <v>90</v>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>Pliegos para regalo del mismo diseño, ideales para tiendas y mesas de regalos.</t>
+          <t>Foami con brillantina que no se cae. Para coronas, letreros y adornos con brillo.</t>
         </is>
       </c>
       <c r="K47" s="5" t="inlineStr">
         <is>
-          <t>Medida del pliego: 70 × 100 cm; Contenido: 25 pliegos</t>
-        </is>
-      </c>
-      <c r="L47" s="3" t="n"/>
-      <c r="M47" s="3" t="inlineStr">
-        <is>
-          <t>Diseño</t>
-        </is>
-      </c>
-      <c r="N47" s="3" t="inlineStr">
-        <is>
-          <t>Cumpleaños, Infantil, Baby, Elegante negro y dorado, Navidad, Amor</t>
-        </is>
-      </c>
+          <t>Medida: Carta (21.5 × 28 cm); Contenido: 5 hojas</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>Dorado, Plateado, Rosa, Rojo, Azul, Morado, Verde</t>
+        </is>
+      </c>
+      <c r="M47" s="3" t="n"/>
+      <c r="N47" s="3" t="n"/>
       <c r="O47" s="3" t="n"/>
       <c r="P47" s="3" t="n"/>
       <c r="Q47" s="3" t="inlineStr">
@@ -5214,7 +5222,7 @@
       </c>
       <c r="T47" s="3" t="inlineStr">
         <is>
-          <t>papel envolver regalo pliegos mayoreo</t>
+          <t>foami diamantado brillantina glitter escarchado</t>
         </is>
       </c>
       <c r="U47" s="3" t="n"/>
@@ -5223,52 +5231,56 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>papel-kraft-rollo-10m</t>
+          <t>papel-metalico-pliego</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Papel kraft, rollo 90 cm × 10 m</t>
+          <t>Papel metálico, pliego 50 × 70 cm</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Envolturas</t>
+          <t>Papelería</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Bodas y aniversarios, Navidad</t>
+          <t>Navidad, Graduación</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>95</v>
+        <v>12</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>82</v>
+        <v>9</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>rollo</t>
+          <t>pliego</t>
         </is>
       </c>
       <c r="I48" s="3" t="n">
-        <v>1100</v>
+        <v>30</v>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>Papel kraft natural para envolturas rústicas, manteles de mesa de postres y empaques.</t>
+          <t>Papel con acabado espejo para forrar cajas, hacer moños y decorar fondos.</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
         <is>
-          <t>Medida: 90 cm × 10 m; Gramaje: 80 g/m²</t>
-        </is>
-      </c>
-      <c r="L48" s="3" t="n"/>
+          <t>Medida: 50 × 70 cm; Acabado: Metálico brillante</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>Dorado, Plateado, Rojo, Verde, Azul, Rosa</t>
+        </is>
+      </c>
       <c r="M48" s="3" t="n"/>
       <c r="N48" s="3" t="n"/>
       <c r="O48" s="3" t="n"/>
@@ -5290,7 +5302,7 @@
       </c>
       <c r="T48" s="3" t="inlineStr">
         <is>
-          <t>papel kraft estraza rustico empaque</t>
+          <t>papel metalico espejo lustre brillante</t>
         </is>
       </c>
       <c r="U48" s="3" t="n"/>
@@ -5299,54 +5311,54 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>mono-grande-bolsa-10</t>
+          <t>topper-feliz-cumple</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Moño grande para regalo, bolsa 10 pzas</t>
+          <t>Topper para pastel "Feliz Cumple"</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Envolturas</t>
+          <t>Papelería</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Navidad, Bodas y aniversarios, Amor y amistad</t>
+          <t>Cumpleaños</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>bolsa con 10 piezas</t>
+          <t>pieza</t>
         </is>
       </c>
       <c r="I49" s="3" t="n">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>Moños de listón satinado ya armados, con adhesivo en la base.</t>
+          <t>Adorno para pastel de cartulina metálica, con palitos para insertar.</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t>Diámetro: 12 cm; Contenido: 10 moños del mismo color</t>
+          <t>Medida: 15 × 12 cm; Material: Cartulina metálica</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>Rojo, Rosa, Dorado, Plateado, Azul, Morado, Blanco, Verde</t>
+          <t>Dorado, Plateado, Oro rosa, Negro</t>
         </is>
       </c>
       <c r="M49" s="3" t="n"/>
@@ -5370,7 +5382,7 @@
       </c>
       <c r="T49" s="3" t="inlineStr">
         <is>
-          <t>moño moños regalo listón adhesivo</t>
+          <t>topper pastel adorno cake</t>
         </is>
       </c>
       <c r="U49" s="3" t="n"/>
@@ -5379,12 +5391,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>mono-estrella-bolsa-50</t>
+          <t>papel-envolver-rollo-5m</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Moño estrella chico, bolsa 50 pzas</t>
+          <t>Papel para envolver, rollo 70 cm × 5 m</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -5394,7 +5406,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Navidad, Cumpleaños</t>
+          <t>Cumpleaños, Fiestas infantiles, Baby shower, Navidad, Amor y amistad, Bodas y aniversarios</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
@@ -5404,45 +5416,49 @@
         <v>38</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>bolsa con 50 piezas</t>
+          <t>rollo</t>
         </is>
       </c>
       <c r="I50" s="3" t="n">
-        <v>120</v>
+        <v>260</v>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>Moño estrella metálico de 6 cm con adhesivo, para regalos pequeños y bolsas.</t>
+          <t>Papel para regalo en rollo con tubo de cartón. Alcanza para envolver de 8 a 10 regalos medianos.</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr">
         <is>
-          <t>Diámetro: 6 cm; Contenido: 50 moños</t>
-        </is>
-      </c>
-      <c r="L50" s="3" t="inlineStr">
-        <is>
-          <t>Dorado, Plateado, Rojo, Verde, Azul, Rosa</t>
-        </is>
-      </c>
-      <c r="M50" s="3" t="n"/>
-      <c r="N50" s="3" t="n"/>
+          <t>Medida: 70 cm × 5 m; Papel: Couché 60 g/m²</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="n"/>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="N50" s="3" t="inlineStr">
+        <is>
+          <t>Cumpleaños, Infantil, Baby, Elegante negro y dorado, Navidad, Amor</t>
+        </is>
+      </c>
       <c r="O50" s="3" t="n"/>
       <c r="P50" s="3" t="n"/>
       <c r="Q50" s="3" t="inlineStr">
         <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R50" s="3" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="R50" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="S50" s="3" t="inlineStr">
         <is>
           <t>Visible</t>
@@ -5450,7 +5466,7 @@
       </c>
       <c r="T50" s="3" t="inlineStr">
         <is>
-          <t>moño estrella chico regalo metalico</t>
+          <t>papel envolver regalo rollo envoltura</t>
         </is>
       </c>
       <c r="U50" s="3" t="n"/>
@@ -5459,12 +5475,12 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>liston-satinado-1in-20m</t>
+          <t>papel-envolver-pliegos-25</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Listón satinado 1", rollo 20 m</t>
+          <t>Papel para envolver, paquete 25 pliegos</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -5474,43 +5490,47 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Bodas y aniversarios, XV años, Navidad, Amor y amistad</t>
+          <t>Cumpleaños, Fiestas infantiles, Baby shower, Navidad, Amor y amistad, Bodas y aniversarios</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>28</v>
+        <v>120</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>22</v>
+        <v>105</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>rollo de 20 m</t>
+          <t>paquete con 25 pliegos</t>
         </is>
       </c>
       <c r="I51" s="3" t="n">
-        <v>75</v>
+        <v>950</v>
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>Listón satinado de doble cara para moños, recuerdos, arreglos florales y envolturas.</t>
+          <t>Pliegos para regalo del mismo diseño, ideales para tiendas y mesas de regalos.</t>
         </is>
       </c>
       <c r="K51" s="5" t="inlineStr">
         <is>
-          <t>Ancho: 1 in (2.5 cm); Largo: 20 m</t>
-        </is>
-      </c>
-      <c r="L51" s="3" t="inlineStr">
-        <is>
-          <t>Rojo, Rosa, Fucsia, Dorado, Plateado, Azul rey, Azul cielo, Verde, Blanco, Negro, Morado, Vino</t>
-        </is>
-      </c>
-      <c r="M51" s="3" t="n"/>
-      <c r="N51" s="3" t="n"/>
+          <t>Medida del pliego: 70 × 100 cm; Contenido: 25 pliegos</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="n"/>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="N51" s="3" t="inlineStr">
+        <is>
+          <t>Cumpleaños, Infantil, Baby, Elegante negro y dorado, Navidad, Amor</t>
+        </is>
+      </c>
       <c r="O51" s="3" t="n"/>
       <c r="P51" s="3" t="n"/>
       <c r="Q51" s="3" t="inlineStr">
@@ -5530,7 +5550,7 @@
       </c>
       <c r="T51" s="3" t="inlineStr">
         <is>
-          <t>liston satinado moño cinta recuerdos</t>
+          <t>papel envolver regalo pliegos mayoreo</t>
         </is>
       </c>
       <c r="U51" s="3" t="n"/>
@@ -5539,12 +5559,12 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>liston-rizar-100m</t>
+          <t>papel-kraft-rollo-10m</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Listón para rizar, rollo 100 m</t>
+          <t>Papel kraft, rollo 90 cm × 10 m</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -5554,41 +5574,37 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Navidad</t>
+          <t>Bodas y aniversarios, Navidad</t>
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>rollo de 100 m</t>
+          <t>rollo</t>
         </is>
       </c>
       <c r="I52" s="3" t="n">
-        <v>90</v>
+        <v>1100</v>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>Listón de rafia que se riza con tijera. Sirve para amarrar globos y decorar regalos.</t>
+          <t>Papel kraft natural para envolturas rústicas, manteles de mesa de postres y empaques.</t>
         </is>
       </c>
       <c r="K52" s="5" t="inlineStr">
         <is>
-          <t>Ancho: 3/16 in (5 mm); Largo: 100 m</t>
-        </is>
-      </c>
-      <c r="L52" s="3" t="inlineStr">
-        <is>
-          <t>Rojo, Rosa, Dorado, Plateado, Azul, Verde, Morado, Blanco</t>
-        </is>
-      </c>
+          <t>Medida: 90 cm × 10 m; Gramaje: 80 g/m²</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="n"/>
       <c r="M52" s="3" t="n"/>
       <c r="N52" s="3" t="n"/>
       <c r="O52" s="3" t="n"/>
@@ -5610,7 +5626,7 @@
       </c>
       <c r="T52" s="3" t="inlineStr">
         <is>
-          <t>liston rizar rafia globos amarrar</t>
+          <t>papel kraft estraza rustico empaque</t>
         </is>
       </c>
       <c r="U52" s="3" t="n"/>
@@ -5619,12 +5635,12 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>bolsa-regalo-mediana</t>
+          <t>mono-grande-bolsa-10</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Bolsa de regalo mediana 26 × 32 cm</t>
+          <t>Moño grande para regalo, bolsa 10 pzas</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -5634,52 +5650,48 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Fiestas infantiles, Baby shower, Navidad, Amor y amistad, Bodas y aniversarios</t>
+          <t>Cumpleaños, Navidad, Bodas y aniversarios, Amor y amistad</t>
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>pieza</t>
+          <t>bolsa con 10 piezas</t>
         </is>
       </c>
       <c r="I53" s="3" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>Bolsa de papel con asas de cordón y refuerzo en la base.</t>
+          <t>Moños de listón satinado ya armados, con adhesivo en la base.</t>
         </is>
       </c>
       <c r="K53" s="5" t="inlineStr">
         <is>
-          <t>Medida: 26 × 32 × 12 cm; Asas: Cordón</t>
-        </is>
-      </c>
-      <c r="L53" s="3" t="n"/>
-      <c r="M53" s="3" t="inlineStr">
-        <is>
-          <t>Diseño</t>
-        </is>
-      </c>
-      <c r="N53" s="3" t="inlineStr">
-        <is>
-          <t>Cumpleaños, Infantil, Baby, Elegante negro y dorado, Navidad, Amor</t>
-        </is>
-      </c>
+          <t>Diámetro: 12 cm; Contenido: 10 moños del mismo color</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>Rojo, Rosa, Dorado, Plateado, Azul, Morado, Blanco, Verde</t>
+        </is>
+      </c>
+      <c r="M53" s="3" t="n"/>
+      <c r="N53" s="3" t="n"/>
       <c r="O53" s="3" t="n"/>
       <c r="P53" s="3" t="n"/>
       <c r="Q53" s="3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="R53" s="3" t="inlineStr">
@@ -5694,7 +5706,7 @@
       </c>
       <c r="T53" s="3" t="inlineStr">
         <is>
-          <t>bolsa regalo mediana asas</t>
+          <t>moño moños regalo listón adhesivo</t>
         </is>
       </c>
       <c r="U53" s="3" t="n"/>
@@ -5703,12 +5715,12 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>bolsa-regalo-grande</t>
+          <t>mono-estrella-bolsa-50</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Bolsa de regalo grande 33 × 45 cm</t>
+          <t>Moño estrella chico, bolsa 50 pzas</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -5718,21 +5730,21 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Fiestas infantiles, Baby shower, Navidad, Amor y amistad, Bodas y aniversarios</t>
+          <t>Navidad, Cumpleaños</t>
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>pieza</t>
+          <t>bolsa con 50 piezas</t>
         </is>
       </c>
       <c r="I54" s="3" t="n">
@@ -5740,25 +5752,21 @@
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>Bolsa grande para peluches, ropa y regalos voluminosos.</t>
+          <t>Moño estrella metálico de 6 cm con adhesivo, para regalos pequeños y bolsas.</t>
         </is>
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>Medida: 33 × 45 × 15 cm; Asas: Cordón</t>
-        </is>
-      </c>
-      <c r="L54" s="3" t="n"/>
-      <c r="M54" s="3" t="inlineStr">
-        <is>
-          <t>Diseño</t>
-        </is>
-      </c>
-      <c r="N54" s="3" t="inlineStr">
-        <is>
-          <t>Cumpleaños, Infantil, Baby, Elegante negro y dorado, Navidad, Amor</t>
-        </is>
-      </c>
+          <t>Diámetro: 6 cm; Contenido: 50 moños</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>Dorado, Plateado, Rojo, Verde, Azul, Rosa</t>
+        </is>
+      </c>
+      <c r="M54" s="3" t="n"/>
+      <c r="N54" s="3" t="n"/>
       <c r="O54" s="3" t="n"/>
       <c r="P54" s="3" t="n"/>
       <c r="Q54" s="3" t="inlineStr">
@@ -5778,7 +5786,7 @@
       </c>
       <c r="T54" s="3" t="inlineStr">
         <is>
-          <t>bolsa regalo grande asas peluche</t>
+          <t>moño estrella chico regalo metalico</t>
         </is>
       </c>
       <c r="U54" s="3" t="n"/>
@@ -5787,12 +5795,12 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>bolsa-celofan-15x25-100</t>
+          <t>liston-satinado-1in-20m</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Bolsa de celofán 15 × 25 cm, paquete 100</t>
+          <t>Listón satinado 1", rollo 20 m</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -5802,37 +5810,41 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Fiestas infantiles, Navidad</t>
+          <t>Bodas y aniversarios, XV años, Navidad, Amor y amistad</t>
         </is>
       </c>
       <c r="E55" s="4" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>paquete con 100 bolsas</t>
+          <t>rollo de 20 m</t>
         </is>
       </c>
       <c r="I55" s="3" t="n">
-        <v>210</v>
+        <v>75</v>
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>Bolsitas transparentes para dulceros, aguinaldos de posada, galletas y recuerdos.</t>
+          <t>Listón satinado de doble cara para moños, recuerdos, arreglos florales y envolturas.</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t>Medida: 15 × 25 cm; Contenido: 100 bolsas</t>
-        </is>
-      </c>
-      <c r="L55" s="3" t="n"/>
+          <t>Ancho: 1 in (2.5 cm); Largo: 20 m</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>Rojo, Rosa, Fucsia, Dorado, Plateado, Azul rey, Azul cielo, Verde, Blanco, Negro, Morado, Vino</t>
+        </is>
+      </c>
       <c r="M55" s="3" t="n"/>
       <c r="N55" s="3" t="n"/>
       <c r="O55" s="3" t="n"/>
@@ -5854,7 +5866,7 @@
       </c>
       <c r="T55" s="3" t="inlineStr">
         <is>
-          <t>bolsa celofan dulcero dulces aguinaldo posada galletas recuerdos</t>
+          <t>liston satinado moño cinta recuerdos</t>
         </is>
       </c>
       <c r="U55" s="3" t="n"/>
@@ -5863,12 +5875,12 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>celofan-rollo-1x20m</t>
+          <t>liston-rizar-100m</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Papel celofán, rollo 1 × 20 m</t>
+          <t>Listón para rizar, rollo 100 m</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -5878,39 +5890,39 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Navidad, Amor y amistad</t>
+          <t>Cumpleaños, Navidad</t>
         </is>
       </c>
       <c r="E56" s="4" t="n">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>rollo</t>
+          <t>rollo de 100 m</t>
         </is>
       </c>
       <c r="I56" s="3" t="n">
-        <v>600</v>
+        <v>90</v>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>Celofán para envolver canastas, arcones, arreglos y ramos.</t>
+          <t>Listón de rafia que se riza con tijera. Sirve para amarrar globos y decorar regalos.</t>
         </is>
       </c>
       <c r="K56" s="5" t="inlineStr">
         <is>
-          <t>Medida: 1 × 20 m; Calibre: Grueso, no se rompe al doblar</t>
+          <t>Ancho: 3/16 in (5 mm); Largo: 100 m</t>
         </is>
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>Transparente, Rojo #e63946, Rosa, Azul, Verde</t>
+          <t>Rojo, Rosa, Dorado, Plateado, Azul, Verde, Morado, Blanco</t>
         </is>
       </c>
       <c r="M56" s="3" t="n"/>
@@ -5934,7 +5946,7 @@
       </c>
       <c r="T56" s="3" t="inlineStr">
         <is>
-          <t>celofan rollo canasta arcon arreglo transparente</t>
+          <t>liston rizar rafia globos amarrar</t>
         </is>
       </c>
       <c r="U56" s="3" t="n"/>
@@ -5943,12 +5955,12 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>caja-regalo-set-3</t>
+          <t>bolsa-regalo-mediana</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Cajas de regalo con tapa, set de 3</t>
+          <t>Bolsa de regalo mediana 26 × 32 cm</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -5958,55 +5970,59 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Navidad, Amor y amistad, Bodas y aniversarios</t>
+          <t>Cumpleaños, Fiestas infantiles, Baby shower, Navidad, Amor y amistad, Bodas y aniversarios</t>
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>85</v>
+        <v>18</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>set de 3 cajas</t>
+          <t>pieza</t>
         </is>
       </c>
       <c r="I57" s="3" t="n">
-        <v>650</v>
+        <v>75</v>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>Tres cajas rígidas con tapa que se guardan una dentro de otra. Incluyen listón decorativo.</t>
+          <t>Bolsa de papel con asas de cordón y refuerzo en la base.</t>
         </is>
       </c>
       <c r="K57" s="5" t="inlineStr">
         <is>
-          <t>Medidas: 25 × 25, 20 × 20 y 15 × 15 cm; Material: Cartón rígido forrado</t>
-        </is>
-      </c>
-      <c r="L57" s="3" t="inlineStr">
-        <is>
-          <t>Rojo, Kraft, Blanco, Rosa, Negro, Azul rey</t>
-        </is>
-      </c>
-      <c r="M57" s="3" t="n"/>
-      <c r="N57" s="3" t="n"/>
+          <t>Medida: 26 × 32 × 12 cm; Asas: Cordón</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="n"/>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="N57" s="3" t="inlineStr">
+        <is>
+          <t>Cumpleaños, Infantil, Baby, Elegante negro y dorado, Navidad, Amor</t>
+        </is>
+      </c>
       <c r="O57" s="3" t="n"/>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="inlineStr">
         <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="R57" s="3" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="R57" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="S57" s="3" t="inlineStr">
         <is>
           <t>Visible</t>
@@ -6014,7 +6030,7 @@
       </c>
       <c r="T57" s="3" t="inlineStr">
         <is>
-          <t>caja cajas regalo tapa set</t>
+          <t>bolsa regalo mediana asas</t>
         </is>
       </c>
       <c r="U57" s="3" t="n"/>
@@ -6023,12 +6039,12 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>papel-seda-24-hojas</t>
+          <t>bolsa-regalo-grande</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Papel seda para regalo, paquete 24 hojas</t>
+          <t>Bolsa de regalo grande 33 × 45 cm</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -6038,43 +6054,47 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Cumpleaños, Baby shower, Bodas y aniversarios</t>
+          <t>Cumpleaños, Fiestas infantiles, Baby shower, Navidad, Amor y amistad, Bodas y aniversarios</t>
         </is>
       </c>
       <c r="E58" s="4" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>paquete con 24 hojas</t>
+          <t>pieza</t>
         </is>
       </c>
       <c r="I58" s="3" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>Papel seda delgado para acomodar dentro de bolsas y cajas de regalo.</t>
+          <t>Bolsa grande para peluches, ropa y regalos voluminosos.</t>
         </is>
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t>Medida: 50 × 70 cm; Contenido: 24 hojas</t>
-        </is>
-      </c>
-      <c r="L58" s="3" t="inlineStr">
-        <is>
-          <t>Rosa pastel, Rosa, Rojo, Dorado, Azul cielo, Lila, Blanco, Negro</t>
-        </is>
-      </c>
-      <c r="M58" s="3" t="n"/>
-      <c r="N58" s="3" t="n"/>
+          <t>Medida: 33 × 45 × 15 cm; Asas: Cordón</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="n"/>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="N58" s="3" t="inlineStr">
+        <is>
+          <t>Cumpleaños, Infantil, Baby, Elegante negro y dorado, Navidad, Amor</t>
+        </is>
+      </c>
       <c r="O58" s="3" t="n"/>
       <c r="P58" s="3" t="n"/>
       <c r="Q58" s="3" t="inlineStr">
@@ -6094,7 +6114,7 @@
       </c>
       <c r="T58" s="3" t="inlineStr">
         <is>
-          <t>papel seda tissue relleno bolsa regalo</t>
+          <t>bolsa regalo grande asas peluche</t>
         </is>
       </c>
       <c r="U58" s="3" t="n"/>
@@ -6103,12 +6123,12 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>relleno-viruta-papel-100g</t>
+          <t>bolsa-celofan-15x25-100</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Relleno de viruta de papel, 100 g</t>
+          <t>Bolsa de celofán 15 × 25 cm, paquete 100</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -6118,41 +6138,37 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Navidad, Amor y amistad, Bodas y aniversarios</t>
+          <t>Cumpleaños, Fiestas infantiles, Navidad</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>bolsa de 100 g</t>
+          <t>paquete con 100 bolsas</t>
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Papel triturado para canastas, cajas de regalo y arcones navideños.</t>
+          <t>Bolsitas transparentes para dulceros, aguinaldos de posada, galletas y recuerdos.</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t>Contenido: 100 g; Material: Papel reciclado</t>
-        </is>
-      </c>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>Kraft, Blanco, Rosa, Rojo, Dorado, Negro, Verde, Azul</t>
-        </is>
-      </c>
+          <t>Medida: 15 × 25 cm; Contenido: 100 bolsas</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="n"/>
       <c r="M59" s="3" t="n"/>
       <c r="N59" s="3" t="n"/>
       <c r="O59" s="3" t="n"/>
@@ -6174,14 +6190,334 @@
       </c>
       <c r="T59" s="3" t="inlineStr">
         <is>
-          <t>viruta relleno papel triturado canasta arcon</t>
+          <t>bolsa celofan dulcero dulces aguinaldo posada galletas recuerdos</t>
         </is>
       </c>
       <c r="U59" s="3" t="n"/>
       <c r="V59" s="3" t="n"/>
     </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>celofan-rollo-1x20m</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Papel celofán, rollo 1 × 20 m</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Envolturas</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Navidad, Amor y amistad</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="F60" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>rollo</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>Celofán para envolver canastas, arcones, arreglos y ramos.</t>
+        </is>
+      </c>
+      <c r="K60" s="5" t="inlineStr">
+        <is>
+          <t>Medida: 1 × 20 m; Calibre: Grueso, no se rompe al doblar</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>Transparente, Rojo #e63946, Rosa, Azul, Verde</t>
+        </is>
+      </c>
+      <c r="M60" s="3" t="n"/>
+      <c r="N60" s="3" t="n"/>
+      <c r="O60" s="3" t="n"/>
+      <c r="P60" s="3" t="n"/>
+      <c r="Q60" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R60" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S60" s="3" t="inlineStr">
+        <is>
+          <t>Visible</t>
+        </is>
+      </c>
+      <c r="T60" s="3" t="inlineStr">
+        <is>
+          <t>celofan rollo canasta arcon arreglo transparente</t>
+        </is>
+      </c>
+      <c r="U60" s="3" t="n"/>
+      <c r="V60" s="3" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>caja-regalo-set-3</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Cajas de regalo con tapa, set de 3</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Envolturas</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Cumpleaños, Navidad, Amor y amistad, Bodas y aniversarios</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>set de 3 cajas</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>650</v>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>Tres cajas rígidas con tapa que se guardan una dentro de otra. Incluyen listón decorativo.</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="inlineStr">
+        <is>
+          <t>Medidas: 25 × 25, 20 × 20 y 15 × 15 cm; Material: Cartón rígido forrado</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>Rojo, Kraft, Blanco, Rosa, Negro, Azul rey</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="n"/>
+      <c r="N61" s="3" t="n"/>
+      <c r="O61" s="3" t="n"/>
+      <c r="P61" s="3" t="n"/>
+      <c r="Q61" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R61" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S61" s="3" t="inlineStr">
+        <is>
+          <t>Visible</t>
+        </is>
+      </c>
+      <c r="T61" s="3" t="inlineStr">
+        <is>
+          <t>caja cajas regalo tapa set</t>
+        </is>
+      </c>
+      <c r="U61" s="3" t="n"/>
+      <c r="V61" s="3" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>papel-seda-24-hojas</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Papel seda para regalo, paquete 24 hojas</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Envolturas</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Cumpleaños, Baby shower, Bodas y aniversarios</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>paquete con 24 hojas</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>Papel seda delgado para acomodar dentro de bolsas y cajas de regalo.</t>
+        </is>
+      </c>
+      <c r="K62" s="5" t="inlineStr">
+        <is>
+          <t>Medida: 50 × 70 cm; Contenido: 24 hojas</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>Rosa pastel, Rosa, Rojo, Dorado, Azul cielo, Lila, Blanco, Negro</t>
+        </is>
+      </c>
+      <c r="M62" s="3" t="n"/>
+      <c r="N62" s="3" t="n"/>
+      <c r="O62" s="3" t="n"/>
+      <c r="P62" s="3" t="n"/>
+      <c r="Q62" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R62" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S62" s="3" t="inlineStr">
+        <is>
+          <t>Visible</t>
+        </is>
+      </c>
+      <c r="T62" s="3" t="inlineStr">
+        <is>
+          <t>papel seda tissue relleno bolsa regalo</t>
+        </is>
+      </c>
+      <c r="U62" s="3" t="n"/>
+      <c r="V62" s="3" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>relleno-viruta-papel-100g</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Relleno de viruta de papel, 100 g</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Envolturas</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Navidad, Amor y amistad, Bodas y aniversarios</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G63" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>bolsa de 100 g</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>Papel triturado para canastas, cajas de regalo y arcones navideños.</t>
+        </is>
+      </c>
+      <c r="K63" s="5" t="inlineStr">
+        <is>
+          <t>Contenido: 100 g; Material: Papel reciclado</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>Kraft, Blanco, Rosa, Rojo, Dorado, Negro, Verde, Azul</t>
+        </is>
+      </c>
+      <c r="M63" s="3" t="n"/>
+      <c r="N63" s="3" t="n"/>
+      <c r="O63" s="3" t="n"/>
+      <c r="P63" s="3" t="n"/>
+      <c r="Q63" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R63" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S63" s="3" t="inlineStr">
+        <is>
+          <t>Visible</t>
+        </is>
+      </c>
+      <c r="T63" s="3" t="inlineStr">
+        <is>
+          <t>viruta relleno papel triturado canasta arcon</t>
+        </is>
+      </c>
+      <c r="U63" s="3" t="n"/>
+      <c r="V63" s="3" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V59"/>
+  <autoFilter ref="A1:V63"/>
   <dataValidations count="8">
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elige una de las categorías de la lista." type="list">
       <formula1>"Globos de foil,Globos de látex,Papelería,Envolturas"</formula1>
@@ -6219,7 +6555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:D58"/>
+  <dimension ref="B1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -6409,450 +6745,466 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="8" t="inlineStr">
+    <row r="28" ht="15" customHeight="1">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>• Dos bolsas del mismo tamaño con distinta cantidad van en filas separadas, por ejemplo 18" (15 pz) y 18" (25 pz).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>• Los productos con "Sempertex" en el nombre o con tonos de la carta muestran el logo de Sempertex y aparecen en la sección "Globos Sempertex".</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Fotos</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>• Crea en Google Drive una carpeta "Fotos tienda" y súbelas ahí. De preferencia cuadradas, de unos 800 × 800 px.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>• Comparte la carpeta como "Cualquier persona con el enlace". Luego, en cada foto: clic derecho → Compartir → Copiar enlace, y pégalo en la columna Foto.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="B32" s="7" t="inlineStr">
         <is>
+          <t>• Crea en Google Drive una carpeta "Fotos tienda" y súbelas ahí. De preferencia cuadradas, de unos 800 × 800 px.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>• Comparte la carpeta como "Cualquier persona con el enlace". Luego, en cada foto: clic derecho → Compartir → Copiar enlace, y pégalo en la columna Foto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="B34" s="7" t="inlineStr">
+        <is>
           <t>• Para una foto distinta por color usa la columna "Fotos por opción":  Dorado = enlace; Plateado = enlace</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="B33" s="7" t="inlineStr">
+    <row r="35" ht="15" customHeight="1">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>• Si un producto no tiene foto, la tienda muestra una ilustración con la leyenda "Imagen ilustrativa".</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="8" t="inlineStr">
+    <row r="37">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>Qué va en cada columna</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="11" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Columna</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>Qué poner</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>Ejemplo</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="B37" s="12" t="inlineStr">
+    <row r="39" ht="60" customHeight="1">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>Código</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>Identificador para el enlace del producto. Opcional: si lo dejas vacío se crea con el nombre. No lo cambies una vez publicado, porque lo usan los carritos y los enlaces compartidos. En un producto con varios tamaños, pon el mismo código en todas sus filas.</t>
         </is>
       </c>
-      <c r="D37" s="13" t="inlineStr">
+      <c r="D39" s="13" t="inlineStr">
         <is>
           <t>globo-foil-estrella-18</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="B38" s="12" t="inlineStr">
+    <row r="40" ht="15" customHeight="1">
+      <c r="B40" s="12" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>Obligatorio. Nombre que ven los clientes.</t>
         </is>
       </c>
-      <c r="D38" s="13" t="inlineStr">
+      <c r="D40" s="13" t="inlineStr">
         <is>
           <t>Globo foil estrella 18"</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>Categoría</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>Obligatorio. Una de: Globos de foil, Globos de látex, Papelería, Envolturas.</t>
-        </is>
-      </c>
-      <c r="D39" s="13" t="inlineStr">
-        <is>
-          <t>Globos de foil</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>Temáticas</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Separadas por comas. Si escribes una que no existe (por ejemplo "Día de las Madres"), la tienda la crea sola.</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="inlineStr">
-        <is>
-          <t>Cumpleaños, Navidad</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>Precio</t>
+          <t>Categoría</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Obligatorio. Precio de menudeo en pesos, solo el número.</t>
+          <t>Obligatorio. Una de: Globos de foil, Globos de látex, Papelería, Envolturas.</t>
         </is>
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>Globos de foil</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="B42" s="12" t="inlineStr">
         <is>
+          <t>Temáticas</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Separadas por comas. Si escribes una que no existe (por ejemplo "Día de las Madres"), la tienda la crea sola.</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>Cumpleaños, Navidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15" customHeight="1">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>Precio</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Obligatorio. Precio de menudeo en pesos, solo el número.</t>
+        </is>
+      </c>
+      <c r="D43" s="13" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="B44" s="12" t="inlineStr">
+        <is>
           <t>Precio mayoreo</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>Precio por unidad al llegar a la cantidad mínima. Déjalo vacío si no hay mayoreo.</t>
         </is>
       </c>
-      <c r="D42" s="13" t="inlineStr">
+      <c r="D44" s="13" t="inlineStr">
         <is>
           <t>17</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>Mayoreo desde</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Cantidad mínima para el precio de mayoreo. Se suman todos los colores del mismo producto.</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="15" customHeight="1">
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>Se vende por</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Cómo se vende. Vacío = "pieza".</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="inlineStr">
-        <is>
-          <t>bolsa con 50 piezas</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Peso (g)</t>
+          <t>Mayoreo desde</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Gramos por unidad vendida. Se usa para calcular el envío; si falta se usan 100 g.</t>
+          <t>Cantidad mínima para el precio de mayoreo. Se suman todos los colores del mismo producto.</t>
         </is>
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="B46" s="12" t="inlineStr">
         <is>
+          <t>Se vende por</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Cómo se vende. Vacío = "pieza".</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="inlineStr">
+        <is>
+          <t>bolsa con 50 piezas</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>Peso (g)</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Gramos por unidad vendida. Se usa para calcular el envío; si falta se usan 100 g.</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1">
+      <c r="B48" s="12" t="inlineStr">
+        <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>Texto de la página del producto.</t>
         </is>
       </c>
-      <c r="D46" s="13" t="inlineStr">
+      <c r="D48" s="13" t="inlineStr">
         <is>
           <t>Estrella metálica de 18 pulgadas…</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="15" customHeight="1">
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>Características</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>Pares "Dato: valor" separados por punto y coma.</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="inlineStr">
-        <is>
-          <t>Medida: 18 in (45 cm); Material: Foil</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t>Colores</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Nombres separados por comas (ver pestaña Listas). Para otro color agrega su código: "Turquesa #1fb5ad".</t>
-        </is>
-      </c>
-      <c r="D48" s="13" t="inlineStr">
-        <is>
-          <t>Dorado, Plateado, Rosa</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="B49" s="12" t="inlineStr">
         <is>
+          <t>Características</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Pares "Dato: valor" separados por punto y coma.</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>Medida: 18 in (45 cm); Material: Foil</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>Colores</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Nombres separados por comas (ver pestaña Listas). Para otro color agrega su código: "Turquesa #1fb5ad".</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>Dorado, Plateado, Rosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15" customHeight="1">
+      <c r="B51" s="12" t="inlineStr">
+        <is>
           <t>Otra opción</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>Otra elección del cliente además del color: Número, Letra, Diseño, Tamaño…</t>
         </is>
       </c>
-      <c r="D49" s="13" t="inlineStr">
+      <c r="D51" s="13" t="inlineStr">
         <is>
           <t>Número</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="15" customHeight="1">
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>Valores de la opción</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Separados por comas. Puedes usar rangos como 0-9 o A-Z.</t>
-        </is>
-      </c>
-      <c r="D50" s="13" t="inlineStr">
-        <is>
-          <t>0-9</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="B51" s="12" t="inlineStr">
-        <is>
-          <t>Foto</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>Enlace de Google Drive de la foto (compartida como "Cualquier persona con el enlace") o nombre de un archivo de la carpeta img. Vacío = ilustración.</t>
-        </is>
-      </c>
-      <c r="D51" s="13" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/…/view</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t>Fotos por opción</t>
+          <t>Valores de la opción</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Una foto por color u opción: "Dorado = enlace; Plateado = enlace".</t>
+          <t>Separados por comas. Puedes usar rangos como 0-9 o A-Z.</t>
         </is>
       </c>
       <c r="D52" s="13" t="inlineStr">
         <is>
-          <t>Dorado = https://drive.google.com/file/d/…</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="15" customHeight="1">
+          <t>0-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>Destacado</t>
+          <t>Foto</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Sí para mostrarlo en "Lo más pedido".</t>
+          <t>Enlace de Google Drive de la foto (compartida como "Cualquier persona con el enlace") o nombre de un archivo de la carpeta img. Vacío = ilustración.</t>
         </is>
       </c>
       <c r="D53" s="13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>https://drive.google.com/file/d/…/view</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Fotos por opción</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Sí para la etiqueta "Nuevo".</t>
+          <t>Una foto por color u opción: "Dorado = enlace; Plateado = enlace".</t>
         </is>
       </c>
       <c r="D54" s="13" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
+          <t>Dorado = https://drive.google.com/file/d/…</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15" customHeight="1">
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Destacado</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Visible, Agotado (se ve pero no se puede comprar) u Oculto (no aparece en la tienda).</t>
+          <t>Sí para mostrarlo en "Lo más pedido".</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
         <is>
-          <t>Visible</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="B56" s="12" t="inlineStr">
         <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Sí para la etiqueta "Nuevo".</t>
+        </is>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Visible, Agotado (se ve pero no se puede comprar) u Oculto (no aparece en la tienda).</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>Visible</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="15" customHeight="1">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
           <t>Palabras para buscar</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>Otras palabras con las que los clientes buscan este producto.</t>
         </is>
       </c>
-      <c r="D56" s="13" t="inlineStr">
+      <c r="D58" s="13" t="inlineStr">
         <is>
           <t>metalico helio estrellas</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="60" customHeight="1">
-      <c r="B57" s="12" t="inlineStr">
+    <row r="59" ht="60" customHeight="1">
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>Presentación</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>Para vender un producto en varios tamaños: haz una fila por tamaño con el MISMO nombre y escribe aquí el tamaño (5", 12", 18"). Cada fila lleva su precio, mayoreo, peso y presentación; en la tienda se ven como un solo producto con selector de tamaño.</t>
         </is>
       </c>
-      <c r="D57" s="13" t="inlineStr">
+      <c r="D59" s="13" t="inlineStr">
         <is>
           <t>12"</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="B58" s="12" t="inlineStr">
+    <row r="60" ht="30" customHeight="1">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>Colores agotados</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Colores o tonos sin existencia, separados por comas (nombres o códigos de la carta). En un producto con tamaños, aplica solo al tamaño de esa fila.</t>
         </is>
       </c>
-      <c r="D58" s="13" t="inlineStr">
+      <c r="D60" s="13" t="inlineStr">
         <is>
           <t>015, 390</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="31">
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B37:D37"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B30:D30"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B20:D20"/>

</xml_diff>